<commit_message>
Data: Pembaruan berkas data Kode Produk
</commit_message>
<xml_diff>
--- a/Kode Produk.xlsx
+++ b/Kode Produk.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kerja\Tanam Duit\TDID\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dicoding\mutualfund-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A90768-EFF2-4D13-843C-FBDE45686FD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{772DF244-753C-4B9E-A7E6-D30852C66E95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2AB041A1-9E7B-4A73-AA66-03E19C49B108}"/>
   </bookViews>
@@ -57,9 +57,6 @@
     <t>GAMA2MXCFLEXIF00</t>
   </si>
   <si>
-    <t>Syailendra Fixed Income Fund - Kelas A</t>
-  </si>
-  <si>
     <t>SYA02FIC01SFIF01</t>
   </si>
   <si>
@@ -75,9 +72,6 @@
     <t>SYA02EQC01EQSE01</t>
   </si>
   <si>
-    <t>Syailendra Sharia Money Market Fund Kelas A</t>
-  </si>
-  <si>
     <t>SYA02MMS01SMMF01</t>
   </si>
   <si>
@@ -93,9 +87,6 @@
     <t>PG003IFCBISN2700</t>
   </si>
   <si>
-    <t>UOBAM ESG PASAR UANG INDONESIA</t>
-  </si>
-  <si>
     <t>PG003MMCUOBPUI00</t>
   </si>
   <si>
@@ -253,6 +244,15 @@
   </si>
   <si>
     <t>Sucorinvest Premium Sovereign Balanced Fund Kelas A</t>
+  </si>
+  <si>
+    <t>UOBAM ESG Pasar Uang Indonesia</t>
+  </si>
+  <si>
+    <t>Syailendra Fixed Income Fund Kelas A</t>
+  </si>
+  <si>
+    <t>Syailendra Sharia Money Market Fund</t>
   </si>
 </sst>
 </file>
@@ -640,10 +640,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -688,258 +688,258 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>16</v>
+        <v>75</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>22</v>
+        <v>73</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B26" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>